<commit_message>
Update PropHit model and live UI data
</commit_message>
<xml_diff>
--- a/outputs/prophit_today.xlsx
+++ b/outputs/prophit_today.xlsx
@@ -2074,7 +2074,7 @@
       </c>
       <c r="GX2" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY2" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="HB2" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC2" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="GX3" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY3" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="HB3" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC3" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="GX4" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY4" t="inlineStr">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="HB4" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC4" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="GX5" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY5" t="inlineStr">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="HB5" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC5" t="inlineStr">
@@ -4734,7 +4734,7 @@
       </c>
       <c r="GX6" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY6" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="HB6" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC6" t="inlineStr">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="GX7" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY7" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="HB7" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC7" t="inlineStr">
@@ -6138,7 +6138,7 @@
       </c>
       <c r="GX8" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY8" t="inlineStr">
@@ -6158,7 +6158,7 @@
       </c>
       <c r="HB8" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC8" t="inlineStr">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="GX9" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY9" t="inlineStr">
@@ -6786,7 +6786,7 @@
       </c>
       <c r="HB9" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC9" t="inlineStr">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="GX10" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY10" t="inlineStr">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="HB10" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC10" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="GX11" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY11" t="inlineStr">
@@ -8116,7 +8116,7 @@
       </c>
       <c r="HB11" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC11" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="GX12" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY12" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="HB12" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC12" t="inlineStr">
@@ -9426,7 +9426,7 @@
       </c>
       <c r="GX13" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY13" t="inlineStr">
@@ -9446,7 +9446,7 @@
       </c>
       <c r="HB13" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC13" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="GX14" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY14" t="inlineStr">
@@ -10148,7 +10148,7 @@
       </c>
       <c r="HB14" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC14" t="inlineStr">
@@ -10830,7 +10830,7 @@
       </c>
       <c r="GX15" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY15" t="inlineStr">
@@ -10850,7 +10850,7 @@
       </c>
       <c r="HB15" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC15" t="inlineStr">
@@ -11458,7 +11458,7 @@
       </c>
       <c r="GX16" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY16" t="inlineStr">
@@ -11478,7 +11478,7 @@
       </c>
       <c r="HB16" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC16" t="inlineStr">
@@ -12160,7 +12160,7 @@
       </c>
       <c r="GX17" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY17" t="inlineStr">
@@ -12180,7 +12180,7 @@
       </c>
       <c r="HB17" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC17" t="inlineStr">
@@ -12862,7 +12862,7 @@
       </c>
       <c r="GX18" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY18" t="inlineStr">
@@ -12882,7 +12882,7 @@
       </c>
       <c r="HB18" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC18" t="inlineStr">
@@ -13490,7 +13490,7 @@
       </c>
       <c r="GX19" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY19" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="HB19" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC19" t="inlineStr">
@@ -14192,7 +14192,7 @@
       </c>
       <c r="GX20" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY20" t="inlineStr">
@@ -14212,7 +14212,7 @@
       </c>
       <c r="HB20" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC20" t="inlineStr">
@@ -14820,7 +14820,7 @@
       </c>
       <c r="GX21" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY21" t="inlineStr">
@@ -14840,7 +14840,7 @@
       </c>
       <c r="HB21" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC21" t="inlineStr">
@@ -15522,7 +15522,7 @@
       </c>
       <c r="GX22" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY22" t="inlineStr">
@@ -15542,7 +15542,7 @@
       </c>
       <c r="HB22" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC22" t="inlineStr">
@@ -16224,7 +16224,7 @@
       </c>
       <c r="GX23" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY23" t="inlineStr">
@@ -16244,7 +16244,7 @@
       </c>
       <c r="HB23" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC23" t="inlineStr">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="GX24" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY24" t="inlineStr">
@@ -16946,7 +16946,7 @@
       </c>
       <c r="HB24" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC24" t="inlineStr">
@@ -17628,7 +17628,7 @@
       </c>
       <c r="GX25" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY25" t="inlineStr">
@@ -17648,7 +17648,7 @@
       </c>
       <c r="HB25" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC25" t="inlineStr">
@@ -18256,7 +18256,7 @@
       </c>
       <c r="GX26" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY26" t="inlineStr">
@@ -18276,7 +18276,7 @@
       </c>
       <c r="HB26" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC26" t="inlineStr">
@@ -18884,7 +18884,7 @@
       </c>
       <c r="GX27" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY27" t="inlineStr">
@@ -18904,7 +18904,7 @@
       </c>
       <c r="HB27" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC27" t="inlineStr">
@@ -19512,7 +19512,7 @@
       </c>
       <c r="GX28" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY28" t="inlineStr">
@@ -19532,7 +19532,7 @@
       </c>
       <c r="HB28" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC28" t="inlineStr">
@@ -20214,7 +20214,7 @@
       </c>
       <c r="GX29" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY29" t="inlineStr">
@@ -20234,7 +20234,7 @@
       </c>
       <c r="HB29" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC29" t="inlineStr">
@@ -20916,7 +20916,7 @@
       </c>
       <c r="GX30" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY30" t="inlineStr">
@@ -20936,7 +20936,7 @@
       </c>
       <c r="HB30" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC30" t="inlineStr">
@@ -21618,7 +21618,7 @@
       </c>
       <c r="GX31" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY31" t="inlineStr">
@@ -21638,7 +21638,7 @@
       </c>
       <c r="HB31" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC31" t="inlineStr">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="GX32" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY32" t="inlineStr">
@@ -22340,7 +22340,7 @@
       </c>
       <c r="HB32" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC32" t="inlineStr">
@@ -23022,7 +23022,7 @@
       </c>
       <c r="GX33" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY33" t="inlineStr">
@@ -23042,7 +23042,7 @@
       </c>
       <c r="HB33" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC33" t="inlineStr">
@@ -23724,7 +23724,7 @@
       </c>
       <c r="GX34" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY34" t="inlineStr">
@@ -23744,7 +23744,7 @@
       </c>
       <c r="HB34" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC34" t="inlineStr">
@@ -24352,7 +24352,7 @@
       </c>
       <c r="GX35" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY35" t="inlineStr">
@@ -24372,7 +24372,7 @@
       </c>
       <c r="HB35" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC35" t="inlineStr">
@@ -25054,7 +25054,7 @@
       </c>
       <c r="GX36" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY36" t="inlineStr">
@@ -25074,7 +25074,7 @@
       </c>
       <c r="HB36" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC36" t="inlineStr">
@@ -25756,7 +25756,7 @@
       </c>
       <c r="GX37" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY37" t="inlineStr">
@@ -25776,7 +25776,7 @@
       </c>
       <c r="HB37" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC37" t="inlineStr">
@@ -26458,7 +26458,7 @@
       </c>
       <c r="GX38" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY38" t="inlineStr">
@@ -26478,7 +26478,7 @@
       </c>
       <c r="HB38" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC38" t="inlineStr">
@@ -27160,7 +27160,7 @@
       </c>
       <c r="GX39" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY39" t="inlineStr">
@@ -27180,7 +27180,7 @@
       </c>
       <c r="HB39" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC39" t="inlineStr">
@@ -27862,7 +27862,7 @@
       </c>
       <c r="GX40" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY40" t="inlineStr">
@@ -27882,7 +27882,7 @@
       </c>
       <c r="HB40" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC40" t="inlineStr">
@@ -28564,7 +28564,7 @@
       </c>
       <c r="GX41" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY41" t="inlineStr">
@@ -28584,7 +28584,7 @@
       </c>
       <c r="HB41" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC41" t="inlineStr">
@@ -29266,7 +29266,7 @@
       </c>
       <c r="GX42" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY42" t="inlineStr">
@@ -29286,7 +29286,7 @@
       </c>
       <c r="HB42" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC42" t="inlineStr">
@@ -29968,7 +29968,7 @@
       </c>
       <c r="GX43" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY43" t="inlineStr">
@@ -29988,7 +29988,7 @@
       </c>
       <c r="HB43" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC43" t="inlineStr">
@@ -30670,7 +30670,7 @@
       </c>
       <c r="GX44" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY44" t="inlineStr">
@@ -30690,7 +30690,7 @@
       </c>
       <c r="HB44" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC44" t="inlineStr">
@@ -31372,7 +31372,7 @@
       </c>
       <c r="GX45" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY45" t="inlineStr">
@@ -31392,7 +31392,7 @@
       </c>
       <c r="HB45" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC45" t="inlineStr">
@@ -32074,7 +32074,7 @@
       </c>
       <c r="GX46" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY46" t="inlineStr">
@@ -32094,7 +32094,7 @@
       </c>
       <c r="HB46" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC46" t="inlineStr">
@@ -32776,7 +32776,7 @@
       </c>
       <c r="GX47" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY47" t="inlineStr">
@@ -32796,7 +32796,7 @@
       </c>
       <c r="HB47" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC47" t="inlineStr">
@@ -33404,7 +33404,7 @@
       </c>
       <c r="GX48" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY48" t="inlineStr">
@@ -33424,7 +33424,7 @@
       </c>
       <c r="HB48" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC48" t="inlineStr">
@@ -34106,7 +34106,7 @@
       </c>
       <c r="GX49" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY49" t="inlineStr">
@@ -34126,7 +34126,7 @@
       </c>
       <c r="HB49" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC49" t="inlineStr">
@@ -34808,7 +34808,7 @@
       </c>
       <c r="GX50" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY50" t="inlineStr">
@@ -34828,7 +34828,7 @@
       </c>
       <c r="HB50" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC50" t="inlineStr">
@@ -35510,7 +35510,7 @@
       </c>
       <c r="GX51" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY51" t="inlineStr">
@@ -35530,7 +35530,7 @@
       </c>
       <c r="HB51" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC51" t="inlineStr">
@@ -36212,7 +36212,7 @@
       </c>
       <c r="GX52" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY52" t="inlineStr">
@@ -36232,7 +36232,7 @@
       </c>
       <c r="HB52" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC52" t="inlineStr">
@@ -36914,7 +36914,7 @@
       </c>
       <c r="GX53" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY53" t="inlineStr">
@@ -36934,7 +36934,7 @@
       </c>
       <c r="HB53" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC53" t="inlineStr">
@@ -37616,7 +37616,7 @@
       </c>
       <c r="GX54" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY54" t="inlineStr">
@@ -37636,7 +37636,7 @@
       </c>
       <c r="HB54" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC54" t="inlineStr">
@@ -38318,7 +38318,7 @@
       </c>
       <c r="GX55" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY55" t="inlineStr">
@@ -38338,7 +38338,7 @@
       </c>
       <c r="HB55" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC55" t="inlineStr">
@@ -39020,7 +39020,7 @@
       </c>
       <c r="GX56" t="inlineStr">
         <is>
-          <t>2026-10-04 02:40:18 AM</t>
+          <t>2026-10-04 11:48:09 AM</t>
         </is>
       </c>
       <c r="GY56" t="inlineStr">
@@ -39040,7 +39040,7 @@
       </c>
       <c r="HB56" t="inlineStr">
         <is>
-          <t>2026-10-04T02:40:18.768935-04:00</t>
+          <t>2026-10-04T11:48:09.675210-04:00</t>
         </is>
       </c>
       <c r="HC56" t="inlineStr">

</xml_diff>